<commit_message>
částečná úprava posílání cmd
</commit_message>
<xml_diff>
--- a/rozložení gui.xlsx
+++ b/rozložení gui.xlsx
@@ -2,20 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucnmuni-my.sharepoint.com/personal/451229_muni_cz/Documents/Plocha/MOJE/GitHub/Plotter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F29C74B4-7BC5-43E2-841D-4CFBB7D485BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{2CE0E18A-18DD-4757-BAB8-F7F56C86FF59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57A30417-2328-45C3-B7EB-C44F9C2E0A2F}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12615" xr2:uid="{B200F512-454A-4327-AAE4-301253FEF5A9}"/>
+    <workbookView xWindow="71903" yWindow="-98" windowWidth="28995" windowHeight="17475" xr2:uid="{B200F512-454A-4327-AAE4-301253FEF5A9}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="51">
   <si>
     <t>Err samples</t>
   </si>
@@ -92,9 +91,6 @@
     <t>ad hoc save</t>
   </si>
   <si>
-    <t>divace adress</t>
-  </si>
-  <si>
     <t>IP:port</t>
   </si>
   <si>
@@ -162,16 +158,53 @@
   </si>
   <si>
     <t>cute packets</t>
+  </si>
+  <si>
+    <t>device 1</t>
+  </si>
+  <si>
+    <t>device 2</t>
+  </si>
+  <si>
+    <t>device 3</t>
+  </si>
+  <si>
+    <t>device 4</t>
+  </si>
+  <si>
+    <t>device 5</t>
+  </si>
+  <si>
+    <t>select all</t>
+  </si>
+  <si>
+    <t>invert selection</t>
+  </si>
+  <si>
+    <t>dvě karty</t>
+  </si>
+  <si>
+    <t>první bude hromadné ovládání, send cmd …</t>
+  </si>
+  <si>
+    <t>druhá - device manager, můžu si vybrat které vlastnosti zařízení můžu ovládat i z první karty</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="238"/>
@@ -186,7 +219,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -209,11 +242,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -223,13 +269,14 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -569,18 +616,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76B2BACE-1A92-40A1-A5B7-A8E5DF352F74}">
-  <dimension ref="A3:M20"/>
+  <dimension ref="A3:O31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="13" width="9.73046875" customWidth="1"/>
-    <col min="14" max="18" width="7" customWidth="1"/>
-    <col min="19" max="19" width="3.796875" customWidth="1"/>
-    <col min="21" max="21" width="6.59765625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="6.53125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7" customWidth="1"/>
+    <col min="17" max="17" width="3.796875" customWidth="1"/>
+    <col min="19" max="19" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="4" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:15" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="4" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -621,7 +670,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -631,20 +680,20 @@
       <c r="C5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-    </row>
-    <row r="6" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+    </row>
+    <row r="6" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
@@ -652,24 +701,21 @@
         <v>6</v>
       </c>
       <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
+      <c r="D6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
-      <c r="K6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    </row>
+    <row r="7" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -686,16 +732,20 @@
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
-    <row r="8" spans="1:13" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
-    <row r="13" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="14" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
+    <row r="8" spans="1:15" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
+    <row r="13" spans="1:15" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="N13">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
@@ -703,166 +753,463 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M14" s="1">
         <v>123</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A15" s="5" t="s">
+      <c r="N14" t="s">
+        <v>46</v>
+      </c>
+      <c r="O14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="3">
+        <v>123</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="3">
+        <v>123</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K15" s="6"/>
+      <c r="L15" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="M15" s="9"/>
+      <c r="N15" t="s">
+        <v>41</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="M16" s="9"/>
+      <c r="N16" t="s">
+        <v>42</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A17" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="6"/>
+      <c r="H17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J17" s="6"/>
+      <c r="K17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M17" s="9"/>
+      <c r="N17" t="s">
+        <v>43</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="L18" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="M18" s="5">
+        <v>123</v>
+      </c>
+      <c r="N18" t="s">
+        <v>44</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="M19" s="1"/>
+      <c r="N19" t="s">
+        <v>45</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="N20" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="O20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="K15" s="5"/>
-      <c r="L15" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="M15" s="8"/>
-    </row>
-    <row r="16" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="M16" s="8"/>
-    </row>
-    <row r="17" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="3">
-        <v>123</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D17" s="3">
-        <v>123</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="M17" s="8"/>
-    </row>
-    <row r="18" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A18" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G18" s="5"/>
-      <c r="H18" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="J18" s="5"/>
-      <c r="K18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="L18" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="M18" s="5"/>
-    </row>
-    <row r="19" spans="1:13" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="5">
-        <v>123</v>
-      </c>
-      <c r="M19" s="5"/>
-    </row>
-    <row r="20" spans="1:13" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
+    </row>
+    <row r="21" spans="1:15" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="D29" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="D30" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="D31" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="L15:M15"/>
+  <mergeCells count="16">
     <mergeCell ref="L16:M16"/>
     <mergeCell ref="L17:M17"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:E16"/>
     <mergeCell ref="D5:M5"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C18:E18"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="H15:I15"/>
     <mergeCell ref="J15:K15"/>
+    <mergeCell ref="L15:M15"/>
   </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100507B4775FAABDF4484C6497A7A26939B" ma:contentTypeVersion="15" ma:contentTypeDescription="Vytvoří nový dokument" ma:contentTypeScope="" ma:versionID="870ec2c05281441111f56d6a1f6aa224">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="317fa241-dc0d-4a19-bd23-9d6e79d0e5eb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6d47826910fc911520b42af59e532d7b" ns3:_="">
+    <xsd:import namespace="317fa241-dc0d-4a19-bd23-9d6e79d0e5eb"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:_activity" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSystemTags" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="317fa241-dc0d-4a19-bd23-9d6e79d0e5eb" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="11" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="13" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="14" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="18" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_activity" ma:index="19" nillable="true" ma:displayName="_activity" ma:hidden="true" ma:internalName="_activity">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSystemTags" ma:index="21" nillable="true" ma:displayName="MediaServiceSystemTags" ma:hidden="true" ma:internalName="MediaServiceSystemTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Typ obsahu"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Nadpis"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="317fa241-dc0d-4a19-bd23-9d6e79d0e5eb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E912AB6-F720-4C4E-84FE-CEB4207AAD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="317fa241-dc0d-4a19-bd23-9d6e79d0e5eb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B69C1D49-933C-4BBF-A8B4-6A1CF53D51B4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6130CBCD-06E4-4ACD-B4B0-E64A3BDD8762}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="317fa241-dc0d-4a19-bd23-9d6e79d0e5eb"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>